<commit_message>
update to b2b client list
</commit_message>
<xml_diff>
--- a/Daily_Stats_L1_Support.xlsx
+++ b/Daily_Stats_L1_Support.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="72">
   <si>
     <t>Type</t>
   </si>
@@ -46,9 +46,6 @@
     <t>Dallas Mavericks Client Support</t>
   </si>
   <si>
-    <t>EuroLeague Client Support</t>
-  </si>
-  <si>
     <t>Ligue 1 Client Support</t>
   </si>
   <si>
@@ -61,9 +58,6 @@
     <t>NESN Client Support</t>
   </si>
   <si>
-    <t>Newcastle United Client Support</t>
-  </si>
-  <si>
     <t>NHRA Client Support</t>
   </si>
   <si>
@@ -79,18 +73,12 @@
     <t>Sky Sport Now Client Support</t>
   </si>
   <si>
-    <t>TNA Plus Client Support</t>
-  </si>
-  <si>
     <t>UEFA TV Client Support</t>
   </si>
   <si>
     <t>UFC Client Support</t>
   </si>
   <si>
-    <t>WNBA League Pass Client Support</t>
-  </si>
-  <si>
     <t>World Rugby Client Support</t>
   </si>
   <si>
@@ -100,40 +88,22 @@
     <t>B2C</t>
   </si>
   <si>
-    <t>BroadwayHD</t>
-  </si>
-  <si>
-    <t>Dallas Mavericks TV</t>
-  </si>
-  <si>
-    <t>Dice Support Tickets</t>
-  </si>
-  <si>
     <t>EuroLeague TV</t>
   </si>
   <si>
     <t>Ligue 1+</t>
   </si>
   <si>
-    <t>PCB Live</t>
-  </si>
-  <si>
     <t>Racer+</t>
   </si>
   <si>
-    <t>Rugbypass.tv</t>
-  </si>
-  <si>
-    <t>SkweekTV</t>
-  </si>
-  <si>
     <t>Sky Sport Now</t>
   </si>
   <si>
     <t>Sportsnet Pittsburgh</t>
   </si>
   <si>
-    <t>SuperLeague+</t>
+    <t>SuperMotocross Video Pass</t>
   </si>
   <si>
     <t>TNA+</t>
@@ -178,21 +148,24 @@
 Tickets</t>
   </si>
   <si>
-    <t>2026-02-12</t>
+    <t>2026-03-07</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>Endeavor Streaming</t>
-  </si>
-  <si>
-    <t>FIH Client Support</t>
+    <t>AMC Shudder Client Support</t>
+  </si>
+  <si>
+    <t>BroadwayHD</t>
   </si>
   <si>
     <t>Carlisle United TV</t>
   </si>
   <si>
+    <t>Dice Support Tickets</t>
+  </si>
+  <si>
     <t>FIH</t>
   </si>
   <si>
@@ -202,10 +175,22 @@
     <t>NZ Rugby</t>
   </si>
   <si>
-    <t>SuperMotocross Video Pass</t>
-  </si>
-  <si>
-    <t>Univision Now</t>
+    <t>Oilers Plus</t>
+  </si>
+  <si>
+    <t>Rugbypass.tv</t>
+  </si>
+  <si>
+    <t>SkweekTV</t>
+  </si>
+  <si>
+    <t>SPURSPLAY</t>
+  </si>
+  <si>
+    <t>SuperLeague+</t>
+  </si>
+  <si>
+    <t>UEFA TV</t>
   </si>
   <si>
     <t>Univision TVE</t>
@@ -232,28 +217,25 @@
     <t>P1</t>
   </si>
   <si>
-    <t>2026-02-12T19:23:03</t>
-  </si>
-  <si>
-    <t>1576469</t>
-  </si>
-  <si>
-    <t>vod appearing as geo-restricted while it is not.</t>
+    <t>2026-03-07T03:07:39</t>
+  </si>
+  <si>
+    <t>1594631</t>
+  </si>
+  <si>
+    <t>P1 – Audio Sync Issue on Shudder TV Live Event (Joe Bob) Across All Platforms</t>
   </si>
   <si>
     <t> </t>
   </si>
   <si>
-    <t>P2</t>
-  </si>
-  <si>
-    <t>2026-02-12T13:25:26</t>
-  </si>
-  <si>
-    <t>1576223</t>
-  </si>
-  <si>
-    <t>P2 Data Ingestion Issue</t>
+    <t>2026-03-07T03:58:20</t>
+  </si>
+  <si>
+    <t>1594646</t>
+  </si>
+  <si>
+    <t>P1 – Fire TV App Crashes / Shudder TV Failing to Load During Live Event</t>
   </si>
 </sst>
 </file>
@@ -357,7 +339,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="4.83984375" customWidth="true" bestFit="true"/>
@@ -384,7 +366,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="n" s="0">
-        <v>53.0</v>
+        <v>21.0</v>
       </c>
     </row>
     <row r="3">
@@ -395,7 +377,7 @@
         <v>5</v>
       </c>
       <c r="C3" t="n" s="0">
-        <v>77.0</v>
+        <v>83.0</v>
       </c>
     </row>
     <row r="4">
@@ -406,7 +388,7 @@
         <v>6</v>
       </c>
       <c r="C4" t="n" s="0">
-        <v>69.0</v>
+        <v>67.0</v>
       </c>
     </row>
     <row r="5">
@@ -417,7 +399,7 @@
         <v>7</v>
       </c>
       <c r="C5" t="n" s="0">
-        <v>3.0</v>
+        <v>5.0</v>
       </c>
     </row>
     <row r="6">
@@ -472,7 +454,7 @@
         <v>12</v>
       </c>
       <c r="C10" t="n" s="0">
-        <v>1.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="11">
@@ -483,7 +465,7 @@
         <v>13</v>
       </c>
       <c r="C11" t="n" s="0">
-        <v>3.0</v>
+        <v>6.0</v>
       </c>
     </row>
     <row r="12">
@@ -494,7 +476,7 @@
         <v>14</v>
       </c>
       <c r="C12" t="n" s="0">
-        <v>6.0</v>
+        <v>3.0</v>
       </c>
     </row>
     <row r="13">
@@ -505,7 +487,7 @@
         <v>15</v>
       </c>
       <c r="C13" t="n" s="0">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
     </row>
     <row r="14">
@@ -516,7 +498,7 @@
         <v>16</v>
       </c>
       <c r="C14" t="n" s="0">
-        <v>7.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="15">
@@ -527,7 +509,7 @@
         <v>17</v>
       </c>
       <c r="C15" t="n" s="0">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="16">
@@ -538,7 +520,7 @@
         <v>18</v>
       </c>
       <c r="C16" t="n" s="0">
-        <v>1.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="17">
@@ -549,7 +531,7 @@
         <v>19</v>
       </c>
       <c r="C17" t="n" s="0">
-        <v>1.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="18">
@@ -560,7 +542,7 @@
         <v>20</v>
       </c>
       <c r="C18" t="n" s="0">
-        <v>35.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="19">
@@ -571,7 +553,7 @@
         <v>21</v>
       </c>
       <c r="C19" t="n" s="0">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="20">
@@ -582,238 +564,128 @@
         <v>22</v>
       </c>
       <c r="C20" t="n" s="0">
-        <v>4.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="0">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="B21" t="s" s="0">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C21" t="n" s="0">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="0">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="B22" t="s" s="0">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C22" t="n" s="0">
-        <v>1.0</v>
+        <v>6.0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="B23" t="s" s="0">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C23" t="n" s="0">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="0">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="B24" t="s" s="0">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C24" t="n" s="0">
-        <v>1.0</v>
+        <v>42.0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="0">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B25" t="s" s="0">
         <v>28</v>
       </c>
       <c r="C25" t="n" s="0">
-        <v>5.0</v>
+        <v>26.0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="0">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B26" t="s" s="0">
         <v>29</v>
       </c>
       <c r="C26" t="n" s="0">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="0">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B27" t="s" s="0">
         <v>30</v>
       </c>
       <c r="C27" t="n" s="0">
-        <v>1.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="0">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B28" t="s" s="0">
         <v>31</v>
       </c>
       <c r="C28" t="n" s="0">
-        <v>3.0</v>
+        <v>33.0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="0">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B29" t="s" s="0">
         <v>32</v>
       </c>
       <c r="C29" t="n" s="0">
-        <v>7.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="0">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B30" t="s" s="0">
         <v>33</v>
       </c>
       <c r="C30" t="n" s="0">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s" s="0">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="B31" t="s" s="0">
         <v>34</v>
       </c>
       <c r="C31" t="n" s="0">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="s" s="0">
-        <v>27</v>
-      </c>
-      <c r="B32" t="s" s="0">
-        <v>35</v>
-      </c>
-      <c r="C32" t="n" s="0">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="s" s="0">
-        <v>27</v>
-      </c>
-      <c r="B33" t="s" s="0">
-        <v>36</v>
-      </c>
-      <c r="C33" t="n" s="0">
-        <v>6.0</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="s" s="0">
-        <v>27</v>
-      </c>
-      <c r="B34" t="s" s="0">
-        <v>37</v>
-      </c>
-      <c r="C34" t="n" s="0">
-        <v>66.0</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="s" s="0">
-        <v>27</v>
-      </c>
-      <c r="B35" t="s" s="0">
-        <v>38</v>
-      </c>
-      <c r="C35" t="n" s="0">
-        <v>13.0</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="s" s="0">
-        <v>27</v>
-      </c>
-      <c r="B36" t="s" s="0">
-        <v>39</v>
-      </c>
-      <c r="C36" t="n" s="0">
-        <v>8.0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="s" s="0">
-        <v>27</v>
-      </c>
-      <c r="B37" t="s" s="0">
-        <v>40</v>
-      </c>
-      <c r="C37" t="n" s="0">
-        <v>8.0</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="s" s="0">
-        <v>27</v>
-      </c>
-      <c r="B38" t="s" s="0">
-        <v>41</v>
-      </c>
-      <c r="C38" t="n" s="0">
-        <v>11.0</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="s" s="0">
-        <v>27</v>
-      </c>
-      <c r="B39" t="s" s="0">
-        <v>42</v>
-      </c>
-      <c r="C39" t="n" s="0">
-        <v>10.0</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="s" s="0">
-        <v>27</v>
-      </c>
-      <c r="B40" t="s" s="0">
-        <v>43</v>
-      </c>
-      <c r="C40" t="n" s="0">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="s" s="0">
-        <v>44</v>
-      </c>
-      <c r="B41" t="s" s="0">
-        <v>44</v>
-      </c>
-      <c r="C41" t="n" s="0">
-        <v>421.0</v>
+        <v>347.0</v>
       </c>
     </row>
   </sheetData>
@@ -828,7 +700,7 @@
   <cols>
     <col min="1" max="1" width="4.83984375" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="10.0390625" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="30.41015625" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="24.49609375" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="10.95703125" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="6.5625" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="6.5625" customWidth="true" bestFit="true"/>
@@ -842,28 +714,28 @@
         <v>0</v>
       </c>
       <c r="B1" t="s" s="5">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="C1" t="s" s="6">
         <v>1</v>
       </c>
       <c r="D1" t="s" s="7">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="E1" t="s" s="8">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="F1" t="s" s="9">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="G1" t="s" s="10">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="H1" t="s" s="11">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="I1" t="s" s="12">
-        <v>51</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2">
@@ -871,28 +743,28 @@
         <v>3</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="C2" t="s" s="0">
         <v>4</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="E2" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="F2" t="n" s="0">
-        <v>2.0</v>
+        <v>5.0</v>
       </c>
       <c r="G2" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="H2" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="I2" t="n" s="0">
-        <v>2.0</v>
+        <v>5.0</v>
       </c>
     </row>
     <row r="3">
@@ -900,28 +772,28 @@
         <v>3</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>5</v>
+        <v>44</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="E3" t="s" s="0">
-        <v>53</v>
-      </c>
-      <c r="F3" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
+      </c>
+      <c r="F3" t="n" s="0">
+        <v>3.0</v>
       </c>
       <c r="G3" t="s" s="0">
-        <v>53</v>
-      </c>
-      <c r="H3" t="n" s="0">
-        <v>1.0</v>
+        <v>43</v>
+      </c>
+      <c r="H3" t="s" s="0">
+        <v>43</v>
       </c>
       <c r="I3" t="n" s="0">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
     </row>
     <row r="4">
@@ -929,28 +801,28 @@
         <v>3</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="C4" t="s" s="0">
         <v>6</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="E4" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="F4" t="n" s="0">
-        <v>6.0</v>
+        <v>2.0</v>
       </c>
       <c r="G4" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="H4" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="I4" t="n" s="0">
-        <v>6.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="5">
@@ -958,28 +830,28 @@
         <v>3</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="F5" t="n" s="0">
-        <v>1.0</v>
+        <v>4.0</v>
       </c>
       <c r="G5" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="H5" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="I5" t="n" s="0">
-        <v>1.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="6">
@@ -987,25 +859,25 @@
         <v>3</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>54</v>
+        <v>21</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="E6" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="F6" t="n" s="0">
         <v>1.0</v>
       </c>
       <c r="G6" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="H6" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="I6" t="n" s="0">
         <v>1.0</v>
@@ -1016,83 +888,83 @@
         <v>3</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="C7" t="s" s="0">
-        <v>55</v>
+        <v>22</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="E7" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="F7" t="n" s="0">
-        <v>1.0</v>
+        <v>9.0</v>
       </c>
       <c r="G7" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="H7" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="I7" t="n" s="0">
-        <v>1.0</v>
+        <v>9.0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="C8" t="s" s="0">
-        <v>13</v>
+        <v>45</v>
       </c>
       <c r="D8" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="E8" t="s" s="0">
-        <v>53</v>
-      </c>
-      <c r="F8" t="n" s="0">
-        <v>1.0</v>
+        <v>43</v>
+      </c>
+      <c r="F8" t="s" s="0">
+        <v>43</v>
       </c>
       <c r="G8" t="s" s="0">
-        <v>53</v>
-      </c>
-      <c r="H8" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
+      </c>
+      <c r="H8" t="n" s="0">
+        <v>4.0</v>
       </c>
       <c r="I8" t="n" s="0">
-        <v>1.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="C9" t="s" s="0">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="D9" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="E9" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="F9" t="n" s="0">
         <v>1.0</v>
       </c>
       <c r="G9" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="H9" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="I9" t="n" s="0">
         <v>1.0</v>
@@ -1100,463 +972,463 @@
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="C10" t="s" s="0">
-        <v>20</v>
+        <v>47</v>
       </c>
       <c r="D10" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="E10" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="F10" t="n" s="0">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="G10" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="H10" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="I10" t="n" s="0">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="C11" t="s" s="0">
-        <v>28</v>
-      </c>
-      <c r="D11" t="s" s="0">
-        <v>53</v>
+        <v>24</v>
+      </c>
+      <c r="D11" t="n" s="0">
+        <v>1.0</v>
       </c>
       <c r="E11" t="s" s="0">
-        <v>53</v>
-      </c>
-      <c r="F11" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
+      </c>
+      <c r="F11" t="n" s="0">
+        <v>46.0</v>
       </c>
       <c r="G11" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="H11" t="n" s="0">
         <v>2.0</v>
       </c>
       <c r="I11" t="n" s="0">
-        <v>2.0</v>
+        <v>49.0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="C12" t="s" s="0">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="D12" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="E12" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="F12" t="n" s="0">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="G12" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="H12" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="I12" t="n" s="0">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="C13" t="s" s="0">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D13" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="E13" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="F13" t="n" s="0">
-        <v>1.0</v>
-      </c>
-      <c r="G13" t="s" s="0">
-        <v>53</v>
-      </c>
-      <c r="H13" t="s" s="0">
-        <v>53</v>
+        <v>268.0</v>
+      </c>
+      <c r="G13" t="n" s="0">
+        <v>40.0</v>
+      </c>
+      <c r="H13" t="n" s="0">
+        <v>6.0</v>
       </c>
       <c r="I13" t="n" s="0">
-        <v>1.0</v>
+        <v>314.0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="C14" t="s" s="0">
-        <v>31</v>
+        <v>49</v>
       </c>
       <c r="D14" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="E14" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="F14" t="n" s="0">
-        <v>62.0</v>
-      </c>
-      <c r="G14" t="n" s="0">
-        <v>15.0</v>
-      </c>
-      <c r="H14" t="n" s="0">
-        <v>3.0</v>
+        <v>1.0</v>
+      </c>
+      <c r="G14" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="H14" t="s" s="0">
+        <v>43</v>
       </c>
       <c r="I14" t="n" s="0">
-        <v>80.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="C15" t="s" s="0">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="D15" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="E15" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="F15" t="n" s="0">
         <v>2.0</v>
       </c>
       <c r="G15" t="s" s="0">
-        <v>53</v>
-      </c>
-      <c r="H15" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
+      </c>
+      <c r="H15" t="n" s="0">
+        <v>1.0</v>
       </c>
       <c r="I15" t="n" s="0">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="C16" t="s" s="0">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="D16" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="E16" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="F16" t="n" s="0">
-        <v>259.0</v>
+        <v>3.0</v>
       </c>
       <c r="G16" t="s" s="0">
-        <v>53</v>
-      </c>
-      <c r="H16" t="n" s="0">
-        <v>5.0</v>
+        <v>43</v>
+      </c>
+      <c r="H16" t="s" s="0">
+        <v>43</v>
       </c>
       <c r="I16" t="n" s="0">
-        <v>264.0</v>
+        <v>3.0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="C17" t="s" s="0">
-        <v>58</v>
+        <v>26</v>
       </c>
       <c r="D17" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="E17" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="F17" t="n" s="0">
         <v>1.0</v>
       </c>
       <c r="G17" t="s" s="0">
-        <v>53</v>
-      </c>
-      <c r="H17" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
+      </c>
+      <c r="H17" t="n" s="0">
+        <v>1.0</v>
       </c>
       <c r="I17" t="n" s="0">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B18" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="C18" t="s" s="0">
         <v>52</v>
       </c>
-      <c r="C18" t="s" s="0">
-        <v>59</v>
-      </c>
       <c r="D18" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="E18" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="F18" t="n" s="0">
-        <v>4.0</v>
+        <v>2.0</v>
       </c>
       <c r="G18" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="H18" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="I18" t="n" s="0">
-        <v>4.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="C19" t="s" s="0">
-        <v>34</v>
+        <v>53</v>
       </c>
       <c r="D19" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="E19" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="F19" t="n" s="0">
-        <v>1.0</v>
+        <v>12.0</v>
       </c>
       <c r="G19" t="s" s="0">
-        <v>53</v>
-      </c>
-      <c r="H19" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
+      </c>
+      <c r="H19" t="n" s="0">
+        <v>3.0</v>
       </c>
       <c r="I19" t="n" s="0">
-        <v>1.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="B20" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="C20" t="s" s="0">
         <v>27</v>
       </c>
-      <c r="B20" t="s" s="0">
-        <v>52</v>
-      </c>
-      <c r="C20" t="s" s="0">
-        <v>36</v>
-      </c>
-      <c r="D20" t="s" s="0">
-        <v>53</v>
+      <c r="D20" t="n" s="0">
+        <v>1.0</v>
       </c>
       <c r="E20" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="F20" t="n" s="0">
-        <v>5.0</v>
-      </c>
-      <c r="G20" t="s" s="0">
-        <v>53</v>
+        <v>53.0</v>
+      </c>
+      <c r="G20" t="n" s="0">
+        <v>78.0</v>
       </c>
       <c r="H20" t="n" s="0">
-        <v>1.0</v>
+        <v>6.0</v>
       </c>
       <c r="I20" t="n" s="0">
-        <v>6.0</v>
+        <v>138.0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="0">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B21" t="s" s="0">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="C21" t="s" s="0">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="D21" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="E21" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="F21" t="n" s="0">
-        <v>69.0</v>
-      </c>
-      <c r="G21" t="n" s="0">
-        <v>30.0</v>
+        <v>27.0</v>
+      </c>
+      <c r="G21" t="s" s="0">
+        <v>43</v>
       </c>
       <c r="H21" t="n" s="0">
-        <v>11.0</v>
+        <v>2.0</v>
       </c>
       <c r="I21" t="n" s="0">
-        <v>110.0</v>
+        <v>29.0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="0">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B22" t="s" s="0">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="C22" t="s" s="0">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="D22" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="E22" t="s" s="0">
-        <v>53</v>
-      </c>
-      <c r="F22" t="n" s="0">
-        <v>9.0</v>
+        <v>43</v>
+      </c>
+      <c r="F22" t="s" s="0">
+        <v>43</v>
       </c>
       <c r="G22" t="s" s="0">
-        <v>53</v>
-      </c>
-      <c r="H22" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
+      </c>
+      <c r="H22" t="n" s="0">
+        <v>1.0</v>
       </c>
       <c r="I22" t="n" s="0">
-        <v>9.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B23" t="s" s="0">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="C23" t="s" s="0">
-        <v>39</v>
+        <v>55</v>
       </c>
       <c r="D23" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="E23" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="F23" t="n" s="0">
-        <v>21.0</v>
+        <v>3.0</v>
       </c>
       <c r="G23" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="H23" t="n" s="0">
         <v>1.0</v>
       </c>
       <c r="I23" t="n" s="0">
-        <v>22.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="0">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B24" t="s" s="0">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="C24" t="s" s="0">
-        <v>60</v>
+        <v>29</v>
       </c>
       <c r="D24" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="E24" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="F24" t="n" s="0">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="G24" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="H24" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="I24" t="n" s="0">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="0">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B25" t="s" s="0">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="C25" t="s" s="0">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="D25" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="E25" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="F25" t="n" s="0">
-        <v>6.0</v>
+        <v>5.0</v>
       </c>
       <c r="G25" t="s" s="0">
-        <v>53</v>
-      </c>
-      <c r="H25" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
+      </c>
+      <c r="H25" t="n" s="0">
+        <v>1.0</v>
       </c>
       <c r="I25" t="n" s="0">
         <v>6.0</v>
@@ -1564,112 +1436,112 @@
     </row>
     <row r="26">
       <c r="A26" t="s" s="0">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B26" t="s" s="0">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="C26" t="s" s="0">
-        <v>41</v>
-      </c>
-      <c r="D26" t="n" s="0">
-        <v>4.0</v>
-      </c>
-      <c r="E26" t="n" s="0">
-        <v>9.0</v>
+        <v>56</v>
+      </c>
+      <c r="D26" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="E26" t="s" s="0">
+        <v>43</v>
       </c>
       <c r="F26" t="n" s="0">
-        <v>22.0</v>
+        <v>1.0</v>
       </c>
       <c r="G26" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="H26" t="n" s="0">
-        <v>14.0</v>
+        <v>1.0</v>
       </c>
       <c r="I26" t="n" s="0">
-        <v>49.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="0">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B27" t="s" s="0">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="C27" t="s" s="0">
-        <v>42</v>
-      </c>
-      <c r="D27" t="s" s="0">
-        <v>53</v>
-      </c>
-      <c r="E27" t="s" s="0">
-        <v>53</v>
+        <v>31</v>
+      </c>
+      <c r="D27" t="n" s="0">
+        <v>3.0</v>
+      </c>
+      <c r="E27" t="n" s="0">
+        <v>39.0</v>
       </c>
       <c r="F27" t="n" s="0">
-        <v>128.0</v>
+        <v>60.0</v>
       </c>
       <c r="G27" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="H27" t="n" s="0">
-        <v>6.0</v>
+        <v>16.0</v>
       </c>
       <c r="I27" t="n" s="0">
-        <v>134.0</v>
+        <v>118.0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="0">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B28" t="s" s="0">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="C28" t="s" s="0">
-        <v>61</v>
+        <v>32</v>
       </c>
       <c r="D28" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="E28" t="s" s="0">
-        <v>53</v>
-      </c>
-      <c r="F28" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
+      </c>
+      <c r="F28" t="n" s="0">
+        <v>6.0</v>
       </c>
       <c r="G28" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="H28" t="n" s="0">
         <v>1.0</v>
       </c>
       <c r="I28" t="n" s="0">
-        <v>1.0</v>
+        <v>7.0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="0">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B29" t="s" s="0">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="C29" t="s" s="0">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="D29" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="E29" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="F29" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="G29" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="H29" t="n" s="0">
         <v>1.0</v>
@@ -1680,60 +1552,60 @@
     </row>
     <row r="30">
       <c r="A30" t="s" s="0">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B30" t="s" s="0">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="C30" t="s" s="0">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="D30" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="E30" t="s" s="0">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="F30" t="n" s="0">
-        <v>4.0</v>
+        <v>15.0</v>
       </c>
       <c r="G30" t="s" s="0">
-        <v>53</v>
-      </c>
-      <c r="H30" t="n" s="0">
-        <v>1.0</v>
+        <v>43</v>
+      </c>
+      <c r="H30" t="s" s="0">
+        <v>43</v>
       </c>
       <c r="I30" t="n" s="0">
-        <v>5.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s" s="0">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="B31" t="s" s="0">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="C31" t="s" s="0">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="D31" t="n" s="0">
-        <v>4.0</v>
+        <v>5.0</v>
       </c>
       <c r="E31" t="n" s="0">
-        <v>9.0</v>
+        <v>39.0</v>
       </c>
       <c r="F31" t="n" s="0">
-        <v>612.0</v>
+        <v>537.0</v>
       </c>
       <c r="G31" t="n" s="0">
-        <v>45.0</v>
+        <v>118.0</v>
       </c>
       <c r="H31" t="n" s="0">
         <v>47.0</v>
       </c>
       <c r="I31" t="n" s="0">
-        <v>717.0</v>
+        <v>746.0</v>
       </c>
     </row>
   </sheetData>
@@ -1749,53 +1621,53 @@
     <col min="1" max="1" width="10.625" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="17.94921875" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="7.9140625" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="30.41015625" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="38.875" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="24.37109375" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="64.27734375" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="15.265625" customWidth="true" bestFit="true"/>
     <col min="7" max="7" width="6.5625" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="13">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="B1" t="s" s="14">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="C1" t="s" s="15">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="D1" t="s" s="16">
         <v>1</v>
       </c>
       <c r="E1" t="s" s="17">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="F1" t="s" s="18">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="G1" t="s" s="19">
-        <v>68</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>5</v>
+        <v>44</v>
       </c>
       <c r="E2" t="s" s="0">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="F2" t="s" s="0">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="G2" t="n" s="0">
         <v>1.0</v>
@@ -1803,22 +1675,22 @@
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>13</v>
+        <v>44</v>
       </c>
       <c r="E3" t="s" s="0">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="F3" t="s" s="0">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="G3" t="n" s="0">
         <v>1.0</v>

</xml_diff>